<commit_message>
modifier selection des rounds
</commit_message>
<xml_diff>
--- a/alpes_roundnet.xlsx
+++ b/alpes_roundnet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="78">
   <si>
     <t>Nom</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t>Paul.D</t>
+  </si>
+  <si>
+    <t>Romain.C</t>
   </si>
 </sst>
 </file>
@@ -1452,7 +1455,7 @@
       </c>
     </row>
     <row r="59" ht="14.25">
-      <c r="A59" s="3" t="s">
+      <c r="A59" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B59">
@@ -1518,7 +1521,7 @@
       </c>
     </row>
     <row r="65" ht="14.25">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="2" t="s">
         <v>68</v>
       </c>
       <c r="B65">
@@ -1551,7 +1554,7 @@
       </c>
     </row>
     <row r="68" ht="14.25">
-      <c r="A68" s="3" t="s">
+      <c r="A68" s="2" t="s">
         <v>71</v>
       </c>
       <c r="B68">
@@ -1562,7 +1565,7 @@
       </c>
     </row>
     <row r="69" ht="14.25">
-      <c r="A69" s="3" t="s">
+      <c r="A69" s="2" t="s">
         <v>72</v>
       </c>
       <c r="B69">
@@ -1573,7 +1576,7 @@
       </c>
     </row>
     <row r="70" ht="14.25">
-      <c r="A70" s="3" t="s">
+      <c r="A70" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B70">
@@ -1584,7 +1587,7 @@
       </c>
     </row>
     <row r="71" ht="14.25">
-      <c r="A71" s="3" t="s">
+      <c r="A71" s="2" t="s">
         <v>74</v>
       </c>
       <c r="B71">
@@ -1595,7 +1598,7 @@
       </c>
     </row>
     <row r="72" ht="14.25">
-      <c r="A72" s="3" t="s">
+      <c r="A72" s="2" t="s">
         <v>75</v>
       </c>
       <c r="B72">
@@ -1606,7 +1609,7 @@
       </c>
     </row>
     <row r="73" ht="14.25">
-      <c r="A73" s="3" t="s">
+      <c r="A73" s="2" t="s">
         <v>76</v>
       </c>
       <c r="B73">
@@ -1617,7 +1620,15 @@
       </c>
     </row>
     <row r="74" ht="14.25">
-      <c r="A74" s="2"/>
+      <c r="A74" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B74">
+        <v>1</v>
+      </c>
+      <c r="C74" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="75" ht="14.25">
       <c r="A75" s="2"/>

</xml_diff>

<commit_message>
ajout des lvl en bye
</commit_message>
<xml_diff>
--- a/alpes_roundnet.xlsx
+++ b/alpes_roundnet.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
   <si>
     <t>Nom</t>
   </si>
@@ -262,6 +262,15 @@
   </si>
   <si>
     <t>vincent.L</t>
+  </si>
+  <si>
+    <t>Archi</t>
+  </si>
+  <si>
+    <t>Chloé</t>
+  </si>
+  <si>
+    <t>Gia</t>
   </si>
 </sst>
 </file>
@@ -1643,7 +1652,7 @@
       </c>
     </row>
     <row r="75" ht="14.25">
-      <c r="A75" s="3" t="s">
+      <c r="A75" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B75">
@@ -1654,7 +1663,7 @@
       </c>
     </row>
     <row r="76" ht="14.25">
-      <c r="A76" s="3" t="s">
+      <c r="A76" s="2" t="s">
         <v>79</v>
       </c>
       <c r="B76">
@@ -1665,7 +1674,7 @@
       </c>
     </row>
     <row r="77" ht="14.25">
-      <c r="A77" s="3" t="s">
+      <c r="A77" s="2" t="s">
         <v>80</v>
       </c>
       <c r="B77">
@@ -1676,7 +1685,7 @@
       </c>
     </row>
     <row r="78" ht="14.25">
-      <c r="A78" s="3" t="s">
+      <c r="A78" s="2" t="s">
         <v>81</v>
       </c>
       <c r="B78">
@@ -1687,13 +1696,37 @@
       </c>
     </row>
     <row r="79" ht="14.25">
-      <c r="A79" s="2"/>
+      <c r="A79" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B79">
+        <v>1</v>
+      </c>
+      <c r="C79" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="80" ht="14.25">
-      <c r="A80" s="2"/>
+      <c r="A80" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B80">
+        <v>2</v>
+      </c>
+      <c r="C80" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="81" ht="14.25">
-      <c r="A81" s="2"/>
+      <c r="A81" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B81">
+        <v>3</v>
+      </c>
+      <c r="C81" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="82" ht="14.25">
       <c r="A82" s="2"/>

</xml_diff>